<commit_message>
feat(idp-studio): add radio toggle stamping, statutory form schema, and deduplicated field editor
</commit_message>
<xml_diff>
--- a/testing/Cameo global/2024-25/Cameo_Global_24_25_AOC4_Populated.xlsx
+++ b/testing/Cameo global/2024-25/Cameo_Global_24_25_AOC4_Populated.xlsx
@@ -348,7 +348,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -492,12 +492,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3227,7 +3231,9 @@
           <t>Turnover @ 10% as per previous year</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n"/>
+      <c r="C6" s="69" t="n">
+        <v>73915481</v>
+      </c>
       <c r="D6" s="14" t="n"/>
       <c r="E6" s="14" t="n"/>
       <c r="F6" s="14" t="n"/>
@@ -3239,7 +3245,9 @@
           <t>Networth @ 10% as per previous year</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n"/>
+      <c r="C7" s="69" t="n">
+        <v>22246914</v>
+      </c>
       <c r="D7" s="14" t="n"/>
       <c r="E7" s="14" t="n"/>
       <c r="F7" s="14" t="n"/>
@@ -3251,11 +3259,11 @@
           <t>If there is Material Transaction, then AOC 2 is applicable. If the transaction is not material AOC 2 is Not applicable</t>
         </is>
       </c>
-      <c r="C8" s="69" t="n"/>
-      <c r="D8" s="69" t="n"/>
-      <c r="E8" s="69" t="n"/>
-      <c r="F8" s="69" t="n"/>
-      <c r="G8" s="69" t="n"/>
+      <c r="C8" s="70" t="n"/>
+      <c r="D8" s="70" t="n"/>
+      <c r="E8" s="70" t="n"/>
+      <c r="F8" s="70" t="n"/>
+      <c r="G8" s="70" t="n"/>
     </row>
     <row r="9" ht="62.4" customHeight="1">
       <c r="B9" s="17" t="inlineStr">
@@ -3501,7 +3509,11 @@
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="22" t="n"/>
       <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
+      <c r="G19" s="59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="28.2" customHeight="1">
       <c r="B20" s="21" t="inlineStr">
@@ -3546,9 +3558,9 @@
           <t>Loans to directors or interested persons of directors</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>APPLICABILITY</t>
+      <c r="D25" s="66" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="E25" s="17" t="inlineStr">
@@ -3568,7 +3580,11 @@
           <t>Has the company given any loan to Directors/ or of a company which is its holding company or any partner or relative of any such director; OR</t>
         </is>
       </c>
-      <c r="D26" s="6" t="n"/>
+      <c r="D26" s="66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E26" s="6" t="n"/>
     </row>
     <row r="27" ht="31.2" customHeight="1">
@@ -3582,7 +3598,11 @@
           <t>Has the company given any loan to any firm in which any such director or relative is a partner</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n"/>
+      <c r="D27" s="66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E27" s="6" t="n"/>
     </row>
     <row r="28" ht="31.2" customHeight="1">
@@ -3608,11 +3628,10 @@
       </c>
       <c r="D29" s="66" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E29" s="6" t="n"/>
-      <c r="F29" s="68" t="inlineStr"/>
     </row>
     <row r="30" ht="46.8" customHeight="1">
       <c r="B30" s="7" t="n"/>
@@ -3621,15 +3640,12 @@
           <t>Its borrowings from banks/financial institutions/any Body Corporate is less than twice of its paid-up share capital or Rs. 50 crore, whichever is lower AND</t>
         </is>
       </c>
-      <c r="D30" s="70" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="D30" s="71" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="E30" s="6" t="n"/>
-      <c r="F30" s="68" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="31" ht="78" customHeight="1">
       <c r="B31" s="7" t="n"/>
@@ -3641,13 +3657,12 @@
 </t>
         </is>
       </c>
-      <c r="D31" s="70" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="D31" s="71" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
       <c r="E31" s="6" t="n"/>
-      <c r="F31" s="68" t="inlineStr"/>
     </row>
     <row r="32" ht="15.6" customHeight="1">
       <c r="B32" s="7" t="n"/>
@@ -3656,8 +3671,8 @@
           <t>Even if one of the above conditions are YES,  Private companies cannot provide loan to its directors or of a company which is its holding company or any partner or relative of any such director</t>
         </is>
       </c>
-      <c r="D32" s="71" t="n"/>
-      <c r="E32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="73" t="n"/>
     </row>
     <row r="33" ht="93.59999999999999" customHeight="1">
       <c r="B33" s="17" t="inlineStr">
@@ -3760,7 +3775,11 @@
           <t>the giving of any loan to a managing or whole-time director</t>
         </is>
       </c>
-      <c r="D42" s="35" t="n"/>
+      <c r="D42" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E42" s="35" t="n"/>
     </row>
     <row r="43" ht="31.2" customHeight="1">
@@ -3770,7 +3789,11 @@
           <t>as a part of the conditions of service extended by the company to all its employees;  or</t>
         </is>
       </c>
-      <c r="D43" s="35" t="n"/>
+      <c r="D43" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E43" s="35" t="n"/>
     </row>
     <row r="44" ht="31.2" customHeight="1">
@@ -3780,7 +3803,11 @@
           <t xml:space="preserve"> pursuant to any scheme approved by the members by a special resolution; </t>
         </is>
       </c>
-      <c r="D44" s="35" t="n"/>
+      <c r="D44" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E44" s="35" t="n"/>
     </row>
     <row r="45" ht="109.2" customHeight="1">
@@ -3790,7 +3817,11 @@
           <t>a company which in the ordinary course of its business provides loans or gives guarantees or securities for the due repayment of any loan and in respect of such loans an interest is charged at a rate not less than the rate of prevailing yield of one year, three year, five year or ten year Government security closest to the tenor of the loan;</t>
         </is>
       </c>
-      <c r="D45" s="35" t="n"/>
+      <c r="D45" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E45" s="35" t="n"/>
     </row>
     <row r="46" ht="78" customHeight="1">
@@ -3800,7 +3831,11 @@
           <t>any loan made by a holding company to its wholly owned subsidiary company or any guarantee given or security provided by a holding company in respect of any loan made to its wholly owned subsidiary company; or</t>
         </is>
       </c>
-      <c r="D46" s="35" t="n"/>
+      <c r="D46" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E46" s="35" t="n"/>
     </row>
     <row r="47" ht="46.8" customHeight="1">
@@ -3810,7 +3845,11 @@
           <t>any guarantee given or security provided by a holding company in respect of loan made by any bank or financial institution to its subsidiary company:</t>
         </is>
       </c>
-      <c r="D47" s="35" t="n"/>
+      <c r="D47" s="74" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E47" s="35" t="n"/>
     </row>
     <row r="48" ht="31.2" customHeight="1">
@@ -3824,7 +3863,11 @@
           <t>Has the Company give loan, guarantee to any person or body corporate</t>
         </is>
       </c>
-      <c r="D48" s="6" t="n"/>
+      <c r="D48" s="66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E48" s="6" t="n"/>
     </row>
     <row r="49" ht="46.8" customHeight="1">
@@ -3838,7 +3881,11 @@
           <t>Has the Company acquired by way of subscription, purchase or otherwise, the securities of any other body corporate,</t>
         </is>
       </c>
-      <c r="D49" s="6" t="n"/>
+      <c r="D49" s="66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E49" s="6" t="n"/>
     </row>
     <row r="50" ht="31.2" customHeight="1">
@@ -3860,13 +3907,10 @@
       </c>
       <c r="D51" s="66" t="inlineStr">
         <is>
-          <t>Applicable</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E51" s="6" t="n"/>
-      <c r="F51" s="68" t="n">
-        <v>162799872</v>
-      </c>
     </row>
     <row r="52" ht="15.6" customHeight="1">
       <c r="B52" s="7" t="n"/>
@@ -3877,13 +3921,10 @@
       </c>
       <c r="D52" s="66" t="inlineStr">
         <is>
-          <t>Applicable</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="E52" s="6" t="n"/>
-      <c r="F52" s="68" t="n">
-        <v>270833120</v>
-      </c>
     </row>
     <row r="53" ht="15.6" customHeight="1">
       <c r="B53" s="7" t="n"/>
@@ -3892,7 +3933,11 @@
           <t>If within limits, include in Board report</t>
         </is>
       </c>
-      <c r="D53" s="6" t="n"/>
+      <c r="D53" s="66" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E53" s="6" t="n"/>
     </row>
     <row r="54" ht="31.2" customHeight="1">
@@ -3902,7 +3947,11 @@
           <t>If exceeding limit, to mention in MGT 8 &amp; prior approval/ratification in next AGM/EGM</t>
         </is>
       </c>
-      <c r="D54" s="6" t="n"/>
+      <c r="D54" s="66" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E54" s="6" t="n"/>
     </row>
   </sheetData>

</xml_diff>